<commit_message>
feat: implement export-to-html functionality for dashboard reports including style inlining and canvas serialization
</commit_message>
<xml_diff>
--- a/tools-platform/backend/templates/每月赛马-分网络.xlsx
+++ b/tools-platform/backend/templates/每月赛马-分网络.xlsx
@@ -115,13 +115,13 @@
     <t>[Map:ORG AOS 2.0过保订单]</t>
   </si>
   <si>
-    <t>VDF: post-warranty order increase with AOS 2.0 package (NetCareEdge and Escape Solution and Network Robustness Assessment - 0.4M)</t>
+    <t>VDF: post-warranty order increase with AOS 2.0 package (NetCareEdge and Escape Solution and Network Robustness Assessment  - 0.4M)</t>
   </si>
   <si>
     <t>[Map:VDF AOS 2.0过保订单]</t>
   </si>
   <si>
-    <t>e&amp; Cost Control: GPR increase 10% to last year</t>
+    <t>e&amp; Cost Control: GPR increase to 20%+</t>
   </si>
   <si>
     <t>[Map:ET成本控制(GPR提升10%)]</t>
@@ -157,7 +157,7 @@
     <t>[Map:全量EOS (合并)]</t>
   </si>
   <si>
-    <t>Urgent EOS Risk: finish the risk mitigation before Nov.(XXXXX)</t>
+    <t>Urgent EOS Risk: finish the risk mitigation before Nov.</t>
   </si>
   <si>
     <t>[Map:重急EOS]</t>
@@ -169,7 +169,7 @@
     <t>[Map:锂电]</t>
   </si>
   <si>
-    <t>Router Rectification: Finish risk clearance on time with high quality</t>
+    <t>Router Rectification:  Finish risk clearance on time with high quality</t>
   </si>
   <si>
     <t>[Map:路由器]</t>
@@ -196,7 +196,7 @@
     <t>[Map:价值网络HC]</t>
   </si>
   <si>
-    <t>Network robustness assessment (ORG and VDF): finish data collection within Apr., finish report to CXO customer within May.</t>
+    <t>Network robustness assessment (ORG and VDF):  finish data collection within Apr., finish report to CXO customer within May.</t>
   </si>
   <si>
     <t>TBD</t>
@@ -223,13 +223,13 @@
     <t>[Map:iLab 应急演练]</t>
   </si>
   <si>
-    <t>Top &amp; Contigency plan update based on HQ regulation (1 time/half year)</t>
+    <t>Top &amp; Contigency plan update based on HQ regulation  (1 time/half year, without overdue)</t>
   </si>
   <si>
     <t>[Map:拓扑与预案 (合并)]</t>
   </si>
   <si>
-    <t>IBMS update based on HQ regulation (1 time/half year)</t>
+    <t>IBMS update based on HQ regulation (1 time/half year, without overdue)</t>
   </si>
   <si>
     <t>[Map:IBMS]</t>
@@ -247,19 +247,19 @@
     <t>Service magazine: 1 time/quarter (submit and archive on Feb.May. Aug. Nov.)</t>
   </si>
   <si>
-    <t>[Map:Jam服务专刊]</t>
+    <t>[Map:Jam服务专刊/季度]</t>
   </si>
   <si>
     <t>Service Summit: 1 time/half year (1: before May., 2: before Nov.)</t>
   </si>
   <si>
-    <t>[Map:服务峰会]</t>
+    <t>[Map:服务峰会/半年]</t>
   </si>
   <si>
     <t>Publish the activity with customer in Jam (1 times/month, more than 1 time add 0.5 extral points)</t>
   </si>
   <si>
-    <t>[Map:Jam客户活动]</t>
+    <t>[Map:Jam客户活动/月度]</t>
   </si>
   <si>
     <t>Capability Improvement</t>
@@ -271,7 +271,7 @@
     <t>[Map:L4骨干]</t>
   </si>
   <si>
-    <t>The average capability score of on-job employees in the CS department is 80 points.</t>
+    <t xml:space="preserve">The average capability score of on-job employees in the CS department is 80 points.  </t>
   </si>
   <si>
     <t>[Map:员工能力]</t>
@@ -307,7 +307,7 @@
     <t>All</t>
   </si>
   <si>
-    <t>1) Man-made Incident (including of incident caused of rectification issue - failed to complete on time, wrongly confirmed as not involved or partial involved)</t>
+    <t>1) Man-made Incident (including of incident caused of rectification issue - failed to complete on time,  wrongly confirmed as not involved or partial involved)</t>
   </si>
   <si>
     <t>10 point/case</t>
@@ -334,7 +334,7 @@
     <t>[Map:严重投诉 (CXO/Operation Head级别)]</t>
   </si>
   <si>
-    <t>4) Major violation found (no report incident and operation without RFC and operate out of MOP) - found by HQ and Region audit</t>
+    <t>4) Major violation found (no report incident and operation without RFC and operate out of MOP) -  found by  HQ and Region audit</t>
   </si>
   <si>
     <t>[Map:严重违规 (瞒报、无方案/越权操作)]</t>
@@ -415,25 +415,25 @@
     <t>2 point/time</t>
   </si>
   <si>
-    <t>[Map:Jam宣传跨及产品逃生演练]</t>
+    <t>[Map:Jam宣传跨及产品逃生演练/半年]</t>
   </si>
   <si>
-    <t>ETAC/GTAC/HQ visiting to show huawei service value (cumulative bonus points)</t>
+    <t>ETAC/GTAC/HQ visiting  to show huawei service value (cumulative bonus points)</t>
   </si>
   <si>
-    <t>[Map:邀约客户交流呈现服务价值]</t>
+    <t>[Map:邀约客户交流呈现服务价值/年度]</t>
   </si>
   <si>
     <t>CS/AMS manager joins spare-parts checks/scrapping/inspection</t>
   </si>
   <si>
-    <t>[Map:CS/AMS主管参与备件盘点/报废/抽检]</t>
+    <t>[Map:CS/AMS主管参与备件盘点/报废/抽检 /月度]</t>
   </si>
   <si>
     <t>On-site SPMS/SPHS presentation</t>
   </si>
   <si>
-    <t>[Map:客户现场宣讲SPMS/SPHS]</t>
+    <t>[Map:客户现场宣讲SPMS/SPHS /月度]</t>
   </si>
   <si>
     <t>[Map:SYS_AdjustTotal]</t>

</xml_diff>

<commit_message>
feat: complete report backup and export handling
</commit_message>
<xml_diff>
--- a/tools-platform/backend/templates/每月赛马-分网络.xlsx
+++ b/tools-platform/backend/templates/每月赛马-分网络.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="148">
   <si>
     <t>Category</t>
   </si>
@@ -271,7 +271,7 @@
     <t>[Map:L4骨干]</t>
   </si>
   <si>
-    <t xml:space="preserve">The average capability score of on-job employees in the CS department is 80 points.  </t>
+    <t>The average capability score of on-job employees in the CS department is 80 points.</t>
   </si>
   <si>
     <t>[Map:员工能力]</t>
@@ -307,7 +307,7 @@
     <t>All</t>
   </si>
   <si>
-    <t>1) Man-made Incident (including of incident caused of rectification issue - failed to complete on time,  wrongly confirmed as not involved or partial involved)</t>
+    <t>Man-made Incident (including of incident caused of rectification issue - failed to complete on time,  wrongly confirmed as not involved or partial involved)</t>
   </si>
   <si>
     <t>10 point/case</t>
@@ -319,7 +319,7 @@
     <t>[Map:人为事故 (含整改逾期、错认漏认)]</t>
   </si>
   <si>
-    <t>2) Incident resore more than 60 mins (Huawei reason)</t>
+    <t>Incident resore more than 60 mins (Huawei reason)</t>
   </si>
   <si>
     <t>5 point/case</t>
@@ -328,13 +328,19 @@
     <t>[Map:恢复超60分钟事故 (华为原因)]</t>
   </si>
   <si>
-    <t>3) Major complains (CXO/Operation Head level) due to CS reason</t>
+    <t>Major complains (CXO/Operation Head level) due to CS reason</t>
   </si>
   <si>
     <t>[Map:严重投诉 (CXO/Operation Head级别)]</t>
   </si>
   <si>
-    <t>4) Major violation found (no report incident and operation without RFC and operate out of MOP) -  found by  HQ and Region audit</t>
+    <t>Incident &amp; High attention issue notice delay</t>
+  </si>
+  <si>
+    <t>[Map:事故与重大问题通报延迟]</t>
+  </si>
+  <si>
+    <t>Major violation found (no report incident and operation without RFC and operate out of MOP) -  found by  HQ and Region audit</t>
   </si>
   <si>
     <t>[Map:严重违规 (瞒报、无方案/越权操作)]</t>
@@ -361,13 +367,13 @@
     <t>[Map:未按要求完成整改 (含延期)]</t>
   </si>
   <si>
-    <t>Non-standard or un-qualified risk handling found in monthly audit</t>
+    <t>Non-standard or un-qualified ticket handling (Risk/SR/others) found in monthly audit</t>
   </si>
   <si>
     <t>2 point/case</t>
   </si>
   <si>
-    <t>[Map:不规范风险处理 (月度审计)]</t>
+    <t>[Map:不规范风险/SR/其它任务处理 (月度审计)]</t>
   </si>
   <si>
     <t>Risk Confirming/Suspend/Close overdue</t>
@@ -409,10 +415,16 @@
     <t>Add</t>
   </si>
   <si>
-    <t>Cross-product contingency plan drills with customers, upload the propaganda in Jam (1 time before May., 1time before Nov.)</t>
+    <t>Others deduction point ( Special scenario based on CSM review )</t>
   </si>
   <si>
     <t>2 point/time</t>
+  </si>
+  <si>
+    <t>[Map:其他扣分项（基于CSM评审的特殊场景）]</t>
+  </si>
+  <si>
+    <t>Cross-product contingency plan drills with customers, upload the propaganda in Jam (1 time before May., 1time before Nov.)</t>
   </si>
   <si>
     <t>[Map:Jam宣传跨及产品逃生演练/半年]</t>
@@ -449,9 +461,6 @@
   </si>
   <si>
     <t>[Map:SYS_FinalResult]</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -2396,7 +2405,7 @@
         <v>105</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E41" s="8" t="s">
         <v>98</v>
@@ -2431,14 +2440,14 @@
       <c r="A42" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B42" s="6">
-        <v>5</v>
+      <c r="B42" s="6" t="s">
+        <v>95</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>107</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="E42" s="8" t="s">
         <v>98</v>
@@ -2450,10 +2459,10 @@
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
       <c r="J42" s="8"/>
-      <c r="K42" s="9"/>
-      <c r="L42" s="9"/>
-      <c r="M42" s="9"/>
-      <c r="N42" s="9"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="8"/>
+      <c r="M42" s="8"/>
+      <c r="N42" s="8"/>
       <c r="O42" s="8"/>
       <c r="P42" s="8"/>
       <c r="Q42" s="8"/>
@@ -2466,7 +2475,7 @@
       <c r="X42" s="1"/>
       <c r="Y42" s="1"/>
       <c r="Z42" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="1:26" x14ac:dyDescent="0.25">
@@ -2477,10 +2486,10 @@
         <v>5</v>
       </c>
       <c r="C43" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="E43" s="8" t="s">
         <v>98</v>
@@ -2522,7 +2531,7 @@
         <v>112</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E44" s="8" t="s">
         <v>98</v>
@@ -2564,7 +2573,7 @@
         <v>114</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E45" s="8" t="s">
         <v>98</v>
@@ -2592,7 +2601,7 @@
       <c r="X45" s="1"/>
       <c r="Y45" s="1"/>
       <c r="Z45" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" spans="1:26" x14ac:dyDescent="0.25">
@@ -2603,10 +2612,10 @@
         <v>5</v>
       </c>
       <c r="C46" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>115</v>
       </c>
       <c r="E46" s="8" t="s">
         <v>98</v>
@@ -2648,7 +2657,7 @@
         <v>119</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E47" s="8" t="s">
         <v>98</v>
@@ -2690,7 +2699,7 @@
         <v>121</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E48" s="8" t="s">
         <v>98</v>
@@ -2732,7 +2741,7 @@
         <v>123</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E49" s="8" t="s">
         <v>98</v>
@@ -2774,7 +2783,7 @@
         <v>125</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>98</v>
@@ -2816,7 +2825,7 @@
         <v>127</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E51" s="8" t="s">
         <v>98</v>
@@ -2849,16 +2858,16 @@
     </row>
     <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B52" s="6">
+        <v>5</v>
+      </c>
+      <c r="C52" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B52" s="6">
-        <v>7</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>130</v>
-      </c>
       <c r="D52" s="8" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="E52" s="8" t="s">
         <v>98</v>
@@ -2886,21 +2895,21 @@
       <c r="X52" s="1"/>
       <c r="Y52" s="1"/>
       <c r="Z52" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B53" s="6">
         <v>10</v>
       </c>
       <c r="C53" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D53" s="8" t="s">
         <v>133</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>131</v>
       </c>
       <c r="E53" s="8" t="s">
         <v>98</v>
@@ -2932,26 +2941,34 @@
       </c>
     </row>
     <row r="54" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="5" t="s">
         <v>135</v>
       </c>
       <c r="B54" s="1"/>
       <c r="C54" s="13"/>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15"/>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="15"/>
-      <c r="N54" s="15"/>
-      <c r="O54" s="15"/>
-      <c r="P54" s="15"/>
-      <c r="Q54" s="15"/>
-      <c r="R54" s="15"/>
+      <c r="F54" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J54" s="8"/>
+      <c r="K54" s="9"/>
+      <c r="L54" s="9"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="9"/>
+      <c r="O54" s="8"/>
+      <c r="P54" s="8"/>
+      <c r="Q54" s="8"/>
+      <c r="R54" s="8"/>
       <c r="S54" s="1"/>
       <c r="T54" s="1"/>
       <c r="U54" s="1"/>
@@ -2964,26 +2981,34 @@
       </c>
     </row>
     <row r="55" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="5" t="s">
         <v>137</v>
       </c>
       <c r="B55" s="1"/>
       <c r="C55" s="13"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
-      <c r="H55" s="15"/>
-      <c r="I55" s="15"/>
-      <c r="J55" s="15"/>
-      <c r="K55" s="15"/>
-      <c r="L55" s="15"/>
-      <c r="M55" s="15"/>
-      <c r="N55" s="15"/>
-      <c r="O55" s="15"/>
-      <c r="P55" s="15"/>
-      <c r="Q55" s="15"/>
-      <c r="R55" s="15"/>
+      <c r="F55" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J55" s="8"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="9"/>
+      <c r="M55" s="9"/>
+      <c r="N55" s="9"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="8"/>
+      <c r="Q55" s="8"/>
+      <c r="R55" s="8"/>
       <c r="S55" s="1"/>
       <c r="T55" s="1"/>
       <c r="U55" s="1"/>
@@ -2997,7 +3022,7 @@
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" s="12" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="B56" s="1"/>
       <c r="C56" s="13"/>
@@ -3024,38 +3049,38 @@
       <c r="X56" s="1"/>
       <c r="Y56" s="1"/>
       <c r="Z56" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="14"/>
-      <c r="J57" s="1"/>
-      <c r="K57" s="14"/>
-      <c r="L57" s="14"/>
-      <c r="M57" s="14"/>
-      <c r="N57" s="14"/>
-      <c r="O57" s="14"/>
-      <c r="P57" s="14"/>
-      <c r="Q57" s="14"/>
-      <c r="R57" s="14"/>
+        <v>141</v>
+      </c>
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
+      <c r="H57" s="15"/>
+      <c r="I57" s="15"/>
+      <c r="J57" s="15"/>
+      <c r="K57" s="15"/>
+      <c r="L57" s="15"/>
+      <c r="M57" s="15"/>
+      <c r="N57" s="15"/>
+      <c r="O57" s="15"/>
+      <c r="P57" s="15"/>
+      <c r="Q57" s="15"/>
+      <c r="R57" s="15"/>
       <c r="S57" s="1"/>
       <c r="T57" s="1"/>
       <c r="U57" s="1"/>
@@ -3064,38 +3089,38 @@
       <c r="X57" s="1"/>
       <c r="Y57" s="1"/>
       <c r="Z57" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58" s="12" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="1"/>
-      <c r="K58" s="14"/>
-      <c r="L58" s="14"/>
-      <c r="M58" s="14"/>
-      <c r="N58" s="14"/>
-      <c r="O58" s="14"/>
-      <c r="P58" s="14"/>
-      <c r="Q58" s="14"/>
-      <c r="R58" s="14"/>
+        <v>92</v>
+      </c>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="15"/>
+      <c r="L58" s="15"/>
+      <c r="M58" s="15"/>
+      <c r="N58" s="15"/>
+      <c r="O58" s="15"/>
+      <c r="P58" s="15"/>
+      <c r="Q58" s="15"/>
+      <c r="R58" s="15"/>
       <c r="S58" s="1"/>
       <c r="T58" s="1"/>
       <c r="U58" s="1"/>
@@ -3108,26 +3133,34 @@
       </c>
     </row>
     <row r="59" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A59" s="16"/>
-      <c r="B59" s="17"/>
+      <c r="A59" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>144</v>
+      </c>
       <c r="C59" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-      <c r="I59" s="1"/>
+      <c r="D59" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F59" s="14"/>
+      <c r="G59" s="14"/>
+      <c r="H59" s="14"/>
+      <c r="I59" s="14"/>
       <c r="J59" s="1"/>
-      <c r="K59" s="1"/>
-      <c r="L59" s="1"/>
-      <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-      <c r="O59" s="1"/>
-      <c r="P59" s="1"/>
-      <c r="Q59" s="1"/>
-      <c r="R59" s="1"/>
+      <c r="K59" s="14"/>
+      <c r="L59" s="14"/>
+      <c r="M59" s="14"/>
+      <c r="N59" s="14"/>
+      <c r="O59" s="14"/>
+      <c r="P59" s="14"/>
+      <c r="Q59" s="14"/>
+      <c r="R59" s="14"/>
       <c r="S59" s="1"/>
       <c r="T59" s="1"/>
       <c r="U59" s="1"/>
@@ -3136,30 +3169,38 @@
       <c r="X59" s="1"/>
       <c r="Y59" s="1"/>
       <c r="Z59" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A60" s="16"/>
-      <c r="B60" s="17"/>
+      <c r="A60" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>146</v>
+      </c>
       <c r="C60" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="1"/>
-      <c r="I60" s="1"/>
+        <v>146</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F60" s="14"/>
+      <c r="G60" s="14"/>
+      <c r="H60" s="14"/>
+      <c r="I60" s="14"/>
       <c r="J60" s="1"/>
-      <c r="K60" s="1"/>
-      <c r="L60" s="1"/>
-      <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
-      <c r="O60" s="1"/>
-      <c r="P60" s="1"/>
-      <c r="Q60" s="1"/>
-      <c r="R60" s="1"/>
+      <c r="K60" s="14"/>
+      <c r="L60" s="14"/>
+      <c r="M60" s="14"/>
+      <c r="N60" s="14"/>
+      <c r="O60" s="14"/>
+      <c r="P60" s="14"/>
+      <c r="Q60" s="14"/>
+      <c r="R60" s="14"/>
       <c r="S60" s="1"/>
       <c r="T60" s="1"/>
       <c r="U60" s="1"/>
@@ -3168,7 +3209,7 @@
       <c r="X60" s="1"/>
       <c r="Y60" s="1"/>
       <c r="Z60" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="61" spans="1:26" x14ac:dyDescent="0.25">

</xml_diff>